<commit_message>
fix(styles): enable to prase color
</commit_message>
<xml_diff>
--- a/example.xlsx
+++ b/example.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\6-market\Market-35a5045b-Luka\rlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{555E7B3E-7313-4B36-887C-98A87B6EF57D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69CC35A5-236A-42CD-9CB2-86B960499F0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="21820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Number" sheetId="1" r:id="rId1"/>
@@ -727,14 +727,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="20.75" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="20.75" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="32.33203125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="32.375" style="1" customWidth="1"/>
     <col min="2" max="2" width="31.5" style="1" customWidth="1"/>
     <col min="3" max="16384" width="20.75" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -742,7 +742,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15.5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>2</v>
       </c>
@@ -750,7 +750,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
@@ -758,7 +758,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -766,7 +766,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>8</v>
       </c>
@@ -786,14 +786,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="20.75" defaultRowHeight="19.899999999999999" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="20.75" defaultRowHeight="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.5" style="5" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" style="5" customWidth="1"/>
+    <col min="2" max="2" width="28.875" style="5" customWidth="1"/>
     <col min="3" max="16384" width="20.75" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>10</v>
       </c>
@@ -801,7 +801,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>12</v>
       </c>
@@ -821,14 +821,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="20.75" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="20.75" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.5" style="5" customWidth="1"/>
     <col min="2" max="2" width="31.5" style="5" customWidth="1"/>
     <col min="3" max="16384" width="20.75" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>14</v>
       </c>
@@ -836,7 +836,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>16</v>
       </c>
@@ -844,7 +844,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>18</v>
       </c>
@@ -852,7 +852,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>20</v>
       </c>
@@ -860,7 +860,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>22</v>
       </c>
@@ -880,12 +880,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="33.5" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="33.5" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="16384" width="33.5" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>24</v>
       </c>
@@ -893,7 +893,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>26</v>
       </c>
@@ -901,7 +901,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>28</v>
       </c>

</xml_diff>